<commit_message>
v4: Improved overall Functionality and added Guideline constraint
</commit_message>
<xml_diff>
--- a/탄소중립_추출결과_20260405_104045.xlsx
+++ b/탄소중립_추출결과_20260405_104045.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/655c961fe41178c9/바탕 화면/과제/4-1/졸업프로젝트/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_AC72E0399969F7C1A8493ABBA91CF68E76692A4A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D18A565E-E23E-4A68-BA51-E6D3AC372BFE}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_AC72E0399969F7C1A8493ABBA91CF68E76692A4A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21788D27-7A6C-4C4C-8665-6F6031AC36C8}"/>
   <bookViews>
-    <workbookView xWindow="6705" yWindow="3405" windowWidth="28800" windowHeight="15345" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="8835" yWindow="2865" windowWidth="28800" windowHeight="15345" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="용도별 자동차(현황)" sheetId="1" r:id="rId1"/>
@@ -3026,11 +3026,15 @@
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
     </font>
     <font>
       <sz val="8"/>
@@ -3143,6 +3147,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -51773,7 +51781,7 @@
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="60" customWidth="1"/>
+    <col min="3" max="3" width="179.125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>